<commit_message>
Actualizacion de la base CRM (captacion de leads)
</commit_message>
<xml_diff>
--- a/Informe_KPIs_CRM_ibis_Styles_Armenia.xlsx
+++ b/Informe_KPIs_CRM_ibis_Styles_Armenia.xlsx
@@ -129,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -144,15 +144,12 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -536,7 +533,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fecha del informe: 17/10/2026</t>
+          <t>Fecha del informe: 19/10/2026</t>
         </is>
       </c>
     </row>
@@ -560,7 +557,7 @@
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Base de datos relacional de ejemplo (200 leads) construida para la sección 7 del plan de marketing del proyecto ibis Styles Armenia. Los datos de personas (nombres, correos, celulares) son 100 % ficticios: se inventaron para demostrar el funcionamiento del CRM. El detalle de la muestra y su justificación están en NOTA_METODOLOGICA_Muestra_CRM.md.</t>
+          <t>Base de datos relacional de ejemplo construida para la sección 7 del plan de marketing del proyecto ibis Styles Armenia. Los datos de personas (nombres, correos, celulares) son 100 % ficticios: se inventaron para demostrar el funcionamiento del CRM. El detalle de la muestra y su justificación están en NOTA_METODOLOGICA_Muestra_CRM.md.</t>
         </is>
       </c>
     </row>
@@ -611,7 +608,7 @@
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>200 leads | 1.156 interacciones | 32 leads calientes | 3 ventas (1.148 COP millones) | 2 opciones en curso | conversión 1,5 % (igual a la meta) | 2 clientes con baja y autorización revocada respetada.</t>
+          <t>Consulte la hoja KPIs para el detalle actualizado.</t>
         </is>
       </c>
     </row>
@@ -641,7 +638,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Operaciones de compraventa (5)</t>
+          <t>Operaciones de compraventa</t>
         </is>
       </c>
     </row>
@@ -652,7 +649,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
+    <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>id_operacion</t>
@@ -690,165 +687,165 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Héctor Duque Herrera</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Promesa</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>2027-03-29</t>
         </is>
       </c>
-      <c r="E5" s="9" t="n">
+      <c r="E5" s="8" t="n">
         <v>374</v>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Piso 4 HAB-07</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>Andrés Giraldo</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Ricardo Montoya Castaño</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Opción</t>
         </is>
       </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>2027-04-28</t>
         </is>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="10" t="n">
         <v>374</v>
       </c>
-      <c r="F6" s="12" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>Piso 7 HAB-02</t>
         </is>
       </c>
-      <c r="G6" s="12" t="inlineStr">
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>Andrés Giraldo</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n">
+      <c r="A7" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Liliana Cardona Orozco</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Promesa</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>2027-05-03</t>
         </is>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="E7" s="8" t="n">
         <v>395</v>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Piso 4 HAB-08</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>Carolina Mejía</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Fernando Quintero Rojas</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Promesa</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>2027-08-12</t>
         </is>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="10" t="n">
         <v>379</v>
       </c>
-      <c r="F8" s="12" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>Piso 12 HAB-02</t>
         </is>
       </c>
-      <c r="G8" s="12" t="inlineStr">
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>Andrés Giraldo</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="n">
+      <c r="A9" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Viviana Zapata Jiménez</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Opción</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>2027-08-26</t>
         </is>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="E9" s="8" t="n">
         <v>402</v>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Piso 13 HAB-09</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>Carolina Mejía</t>
         </is>
@@ -892,7 +889,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
+    <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Alerta</t>
@@ -915,76 +912,76 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>No contactar (baja/revocada)</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="8" t="n">
         <v>65</v>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Juan Salazar Cardona</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>2027-03-25</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>No contactar (baja/revocada)</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="10" t="n">
         <v>186</v>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Ricardo Carlos Vargas Restrepo</t>
         </is>
       </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>2027-10-10</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Leads calificados sin asesor</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Revisar asignación en el CRM</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr"/>
+      <c r="D7" s="8" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Interacciones con fecha inválida</t>
         </is>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Ninguna: todas posteriores al registro</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr"/>
+      <c r="D8" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1021,11 +1018,11 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Los valores corresponden a la base de ejemplo: una muestra; las metas son del plan a 12 meses.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
+          <t>Los valores corresponden a la base: una muestra; las metas son del plan a 12 meses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>KPI</t>
@@ -1041,7 +1038,7 @@
           <t>Meta del plan</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
@@ -1053,76 +1050,76 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Leads en la base</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="8" t="n">
         <v>200</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="8" t="n">
         <v>6000</v>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Por debajo de la meta (muestra)</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Base de ejemplo (muestra para el ejercicio); meta anual del plan: 6.000</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Suites vendidas</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Por debajo de la meta (muestra)</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>Muestra de ejemplo; meta del plan: 90 suites en 12 meses</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Conversión lead a venta</t>
         </is>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="11" t="n">
         <v>0.015</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="8" t="n">
         <v>0.015</v>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Cumple</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Alineada con la meta del plan (1,5%)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Leads por referidos</t>
         </is>
@@ -1130,61 +1127,61 @@
       <c r="B8" s="13" t="n">
         <v>0.095</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="10" t="n">
         <v>0.1</v>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Por debajo de la meta (muestra)</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>9,5% vs meta 10%: muy cerca</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Clientes con autorización vigente o revocada documentada</t>
         </is>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Cumple</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>100% de clientes con consentimiento documentado (Ley 1581)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Valor vendido (COP millones)</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n">
+      <c r="B10" s="10" t="n">
         <v>1148</v>
       </c>
-      <c r="C10" s="12" t="n"/>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Informativo</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>3 promesas de compraventa + 2 opciones en curso</t>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Promesas/escrituras + opciones en curso</t>
         </is>
       </c>
     </row>
@@ -1223,11 +1220,11 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Meta del plan: 1.000 leads/mes (6.000 en 12 meses). La base es una muestra de 200 leads.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
+          <t>Meta del plan: 1.000 leads/mes (6.000 en 12 meses). La base es una muestra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>orden</t>
@@ -1255,30 +1252,30 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Lead</t>
         </is>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="8" t="n">
         <v>200</v>
       </c>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="11" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Lead calificado (MQL)</t>
         </is>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="10" t="n">
         <v>80</v>
       </c>
       <c r="D6" s="13" t="n">
@@ -1289,34 +1286,34 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n">
+      <c r="A7" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Oportunidad (SQL)</t>
         </is>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="11" t="n">
         <v>0.5</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="11" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Reunión o visita</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="10" t="n">
         <v>20</v>
       </c>
       <c r="D8" s="13" t="n">
@@ -1327,34 +1324,34 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="n">
+      <c r="A9" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Opción o separación</t>
         </is>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="11" t="n">
         <v>0.25</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="11" t="n">
         <v>0.25</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Venta</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="10" t="n">
         <v>3</v>
       </c>
       <c r="D10" s="13" t="n">
@@ -1379,7 +1376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -1399,11 +1396,11 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Conversión = ventas / leads del canal. En la muestra, las 3 ventas llegaron por Digital.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
+          <t>Conversión = ventas / leads del canal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>canal</t>
@@ -1431,80 +1428,97 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Digital</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="8" t="n">
         <v>114</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="8" t="n">
         <v>52</v>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="14" t="n">
         <v>0.0263</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Eventos</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Referidos</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="8" t="n">
         <v>19</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Alianzas y relaciones públicas</t>
         </is>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="10" t="n">
         <v>34</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="16" t="n">
+      <c r="E8" s="15" t="n">
         <v>0</v>
       </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>WhatsApp</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="14" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1546,7 +1560,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
+    <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>segmento</t>
@@ -1579,112 +1593,112 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>A. Profesional o empresario urbano</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="8" t="n">
         <v>36</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="8" t="n">
         <v>80</v>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="E5" s="9" t="n">
+      <c r="E5" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="9" t="n">
+      <c r="F5" s="8" t="n">
         <v>395</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>B. Inversionista regional</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="10" t="n">
         <v>22</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>C. Colombianos en el exterior</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="E7" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F7" s="8" t="n">
         <v>379</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>D. Comprador multi-suite</t>
         </is>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="12" t="n">
+      <c r="F8" s="10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>E. Planeación patrimonial</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="E9" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="9" t="n">
+      <c r="F9" s="8" t="n">
         <v>374</v>
       </c>
     </row>
@@ -1729,7 +1743,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
+    <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>campana</t>
@@ -1767,127 +1781,127 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Fase 0. Preparación</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="8" t="n">
         <v>160</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="8" t="n">
         <v>400</v>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="E5" s="9" t="n">
+      <c r="E5" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="9" t="n">
+      <c r="F5" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="G5" s="9" t="n">
+      <c r="G5" s="8" t="n">
         <v>26.7</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>C1. Lanzamiento</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="10" t="n">
         <v>330</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="10" t="n">
         <v>2000</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="10" t="n">
         <v>23</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="10" t="n">
         <v>14.3</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>C2. Conoce tu suite</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="8" t="n">
         <v>290</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="8" t="n">
         <v>1200</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="E7" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F7" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="G7" s="9" t="n">
+      <c r="G7" s="8" t="n">
         <v>11.6</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>C3. Colombia te espera</t>
         </is>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="10" t="n">
         <v>150</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="10" t="n">
         <v>1000</v>
       </c>
-      <c r="D8" s="12" t="n">
+      <c r="D8" s="10" t="n">
         <v>29</v>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="12" t="n">
+      <c r="F8" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="10" t="n">
         <v>10.7</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>C4. Últimos pisos</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="8" t="n">
         <v>220</v>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="8" t="n">
         <v>1400</v>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="8" t="n">
         <v>42</v>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="E9" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="9" t="n">
+      <c r="F9" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="G9" s="9" t="n">
+      <c r="G9" s="8" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1918,7 +1932,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Inventario de 180 suites por estado</t>
+          <t>Inventario de suites por estado</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1943,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
+    <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>estado</t>
@@ -1952,50 +1966,50 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="8" t="n">
         <v>175</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="8" t="n">
         <v>69623.5</v>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="8" t="n">
         <v>397.8</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Separada</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="10" t="n">
         <v>776</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="10" t="n">
         <v>388</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Vendida</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="8" t="n">
         <v>1148</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="8" t="n">
         <v>382.7</v>
       </c>
     </row>
@@ -2036,7 +2050,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
+    <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>clasificacion</t>
@@ -2054,25 +2068,25 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="11" t="n">
         <v>0.01</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Caliente</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="10" t="n">
         <v>32</v>
       </c>
       <c r="C6" s="13" t="n">
@@ -2080,25 +2094,25 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Frío</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="8" t="n">
         <v>77</v>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="11" t="n">
         <v>0.385</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Tibio</t>
         </is>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="10" t="n">
         <v>89</v>
       </c>
       <c r="C8" s="13" t="n">
@@ -2133,7 +2147,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Leads calientes: llamar primero (top 32)</t>
+          <t>Leads calientes: llamar primero</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2158,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
+    <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>cliente</t>
@@ -2172,800 +2186,800 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Daniel Gómez Salazar</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Reunión o visita</t>
         </is>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="8" t="n">
         <v>125</v>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>2027-03-18</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Néstor Ricardo Jiménez Valencia</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Oportunidad (SQL)</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>105</v>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>2027-03-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Camila Henao Salazar</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Reunión o visita</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>2027-03-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Ricardo Montoya Castaño</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Opción o separación</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>105</v>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>2027-04-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Daniel Mejía Torres</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Reunión o visita</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>2027-05-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Marcela Mónica Gómez Martínez</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Reunión o visita</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>105</v>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>2027-05-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Viviana Montoya Cardona</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Reunión o visita</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>2027-07-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Fernando Quintero Rojas</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Venta</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>105</v>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>2027-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Viviana Zapata Jiménez</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Opción o separación</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>2027-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Julián Bedoya Cardona</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Reunión o visita</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>105</v>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>2027-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Héctor Duque Herrera</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Venta</t>
         </is>
       </c>
-      <c r="D6" s="12" t="n">
-        <v>105</v>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>2027-03-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Néstor Ricardo Jiménez Valencia</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="D15" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>2027-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Laura Restrepo Jiménez</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Reunión o visita</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>2027-04-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Iván Duque Ramírez</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Reunión o visita</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>2027-07-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Esteban Juan Betancur Montoya</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Reunión o visita</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>2027-01-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Gustavo Salazar Salazar</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Reunión o visita</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>2027-03-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Camilo Orozco Patiño</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Reunión o visita</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>2027-06-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Claudia Moreno Betancur</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Reunión o visita</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>2027-07-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Diana Liliana Gil Londoño</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Reunión o visita</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>2027-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Sebastián Alejandro Salazar Jiménez</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Oportunidad (SQL)</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
-        <v>105</v>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>2027-03-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Camila Henao Salazar</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="D23" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>2027-03-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Andrea Acosta Orozco</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Oportunidad (SQL)</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>2027-03-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Liliana Cardona Orozco</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Venta</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>2027-04-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Juan Rojas Restrepo</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>Oportunidad (SQL)</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>2027-04-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>Esteban Restrepo Giraldo</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Oportunidad (SQL)</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>2027-04-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Andrés Valencia Bedoya</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Oportunidad (SQL)</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>2027-04-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>Ricardo Camilo Ruiz Cárdenas</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Oportunidad (SQL)</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>2027-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Carolina Viviana Correa Ríos</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>Oportunidad (SQL)</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>2027-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Diego Jorge Cárdenas Londoño</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Reunión o visita</t>
         </is>
       </c>
-      <c r="D8" s="12" t="n">
-        <v>105</v>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>2027-03-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>Ricardo Montoya Castaño</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="D31" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>2027-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>Diego Franco Duque</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>Oportunidad (SQL)</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="n">
+        <v>85</v>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Daniel Martínez Patiño</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Oportunidad (SQL)</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>2027-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>Felipe Felipe Patiño Martínez</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Opción o separación</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="n">
-        <v>105</v>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>2027-04-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Daniel Mejía Torres</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>Reunión o visita</t>
         </is>
       </c>
-      <c r="D10" s="12" t="n">
-        <v>105</v>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>2027-05-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>Marcela Mónica Gómez Martínez</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Reunión o visita</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="n">
-        <v>105</v>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>2027-05-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>Viviana Montoya Cardona</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="D34" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>2027-10-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>Héctor Martínez Duque</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>Reunión o visita</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="n">
-        <v>105</v>
-      </c>
-      <c r="E12" s="12" t="inlineStr">
-        <is>
-          <t>2027-07-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Fernando Quintero Rojas</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>Venta</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="n">
-        <v>105</v>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>2027-08-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>Viviana Zapata Jiménez</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>Opción o separación</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="n">
-        <v>105</v>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>2027-08-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Julián Bedoya Cardona</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>Reunión o visita</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="n">
-        <v>105</v>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>2027-10-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>Laura Restrepo Jiménez</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>Reunión o visita</t>
-        </is>
-      </c>
-      <c r="D16" s="12" t="n">
-        <v>100</v>
-      </c>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>2027-04-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>Iván Duque Ramírez</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Reunión o visita</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="n">
-        <v>100</v>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>2027-07-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Esteban Juan Betancur Montoya</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="inlineStr">
-        <is>
-          <t>Reunión o visita</t>
-        </is>
-      </c>
-      <c r="D18" s="12" t="n">
-        <v>95</v>
-      </c>
-      <c r="E18" s="12" t="inlineStr">
-        <is>
-          <t>2027-01-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>Gustavo Salazar Salazar</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Lead calificado (MQL)</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>2026-11-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Paola Diana Martínez Salazar</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>Reunión o visita</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="n">
-        <v>95</v>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t>2027-03-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Camilo Orozco Patiño</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="inlineStr">
-        <is>
-          <t>Reunión o visita</t>
-        </is>
-      </c>
-      <c r="D20" s="12" t="n">
-        <v>95</v>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>2027-06-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>Claudia Moreno Betancur</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>Reunión o visita</t>
-        </is>
-      </c>
-      <c r="D21" s="9" t="n">
-        <v>95</v>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>2027-07-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>Diana Liliana Gil Londoño</t>
-        </is>
-      </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C22" s="12" t="inlineStr">
-        <is>
-          <t>Reunión o visita</t>
-        </is>
-      </c>
-      <c r="D22" s="12" t="n">
-        <v>95</v>
-      </c>
-      <c r="E22" s="12" t="inlineStr">
-        <is>
-          <t>2027-10-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>Sebastián Alejandro Salazar Jiménez</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>Oportunidad (SQL)</t>
         </is>
       </c>
-      <c r="D23" s="9" t="n">
-        <v>90</v>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>2027-03-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>Andrea Acosta Orozco</t>
-        </is>
-      </c>
-      <c r="B24" s="12" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C24" s="12" t="inlineStr">
-        <is>
-          <t>Oportunidad (SQL)</t>
-        </is>
-      </c>
-      <c r="D24" s="12" t="n">
-        <v>90</v>
-      </c>
-      <c r="E24" s="12" t="inlineStr">
-        <is>
-          <t>2027-03-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>Liliana Cardona Orozco</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Venta</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="n">
-        <v>90</v>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <t>2027-04-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Juan Rojas Restrepo</t>
-        </is>
-      </c>
-      <c r="B26" s="12" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C26" s="12" t="inlineStr">
-        <is>
-          <t>Oportunidad (SQL)</t>
-        </is>
-      </c>
-      <c r="D26" s="12" t="n">
-        <v>90</v>
-      </c>
-      <c r="E26" s="12" t="inlineStr">
-        <is>
-          <t>2027-04-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>Esteban Restrepo Giraldo</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>Oportunidad (SQL)</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="n">
-        <v>90</v>
-      </c>
-      <c r="E27" s="9" t="inlineStr">
-        <is>
-          <t>2027-04-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>Andrés Valencia Bedoya</t>
-        </is>
-      </c>
-      <c r="B28" s="12" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="C28" s="12" t="inlineStr">
-        <is>
-          <t>Oportunidad (SQL)</t>
-        </is>
-      </c>
-      <c r="D28" s="12" t="n">
-        <v>90</v>
-      </c>
-      <c r="E28" s="12" t="inlineStr">
-        <is>
-          <t>2027-04-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>Ricardo Camilo Ruiz Cárdenas</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>Oportunidad (SQL)</t>
-        </is>
-      </c>
-      <c r="D29" s="9" t="n">
-        <v>90</v>
-      </c>
-      <c r="E29" s="9" t="inlineStr">
-        <is>
-          <t>2027-08-27</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
-        <is>
-          <t>Carolina Viviana Correa Ríos</t>
-        </is>
-      </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="inlineStr">
-        <is>
-          <t>Oportunidad (SQL)</t>
-        </is>
-      </c>
-      <c r="D30" s="12" t="n">
-        <v>90</v>
-      </c>
-      <c r="E30" s="12" t="inlineStr">
-        <is>
-          <t>2027-08-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>Diego Jorge Cárdenas Londoño</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>Reunión o visita</t>
-        </is>
-      </c>
-      <c r="D31" s="9" t="n">
-        <v>90</v>
-      </c>
-      <c r="E31" s="9" t="inlineStr">
-        <is>
-          <t>2027-10-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="12" t="inlineStr">
-        <is>
-          <t>Diego Franco Duque</t>
-        </is>
-      </c>
-      <c r="B32" s="12" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C32" s="12" t="inlineStr">
-        <is>
-          <t>Oportunidad (SQL)</t>
-        </is>
-      </c>
-      <c r="D32" s="12" t="n">
-        <v>85</v>
-      </c>
-      <c r="E32" s="12" t="inlineStr">
-        <is>
-          <t>2026-12-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="9" t="inlineStr">
-        <is>
-          <t>Daniel Martínez Patiño</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>Oportunidad (SQL)</t>
-        </is>
-      </c>
-      <c r="D33" s="9" t="n">
-        <v>80</v>
-      </c>
-      <c r="E33" s="9" t="inlineStr">
-        <is>
-          <t>2027-05-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="12" t="inlineStr">
-        <is>
-          <t>Felipe Felipe Patiño Martínez</t>
-        </is>
-      </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C34" s="12" t="inlineStr">
-        <is>
-          <t>Reunión o visita</t>
-        </is>
-      </c>
-      <c r="D34" s="12" t="n">
-        <v>80</v>
-      </c>
-      <c r="E34" s="12" t="inlineStr">
-        <is>
-          <t>2027-10-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="9" t="inlineStr">
-        <is>
-          <t>Héctor Martínez Duque</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>Lead calificado (MQL)</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="n">
+      <c r="D36" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>2026-11-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="12" t="inlineStr">
-        <is>
-          <t>Paola Diana Martínez Salazar</t>
-        </is>
-      </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C36" s="12" t="inlineStr">
-        <is>
-          <t>Oportunidad (SQL)</t>
-        </is>
-      </c>
-      <c r="D36" s="12" t="n">
-        <v>70</v>
-      </c>
-      <c r="E36" s="12" t="inlineStr">
+      <c r="E36" s="10" t="inlineStr">
         <is>
           <t>2027-09-02</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion de la base CRM (inventario vendida 3->2, suite 370M)
</commit_message>
<xml_diff>
--- a/Informe_KPIs_CRM_ibis_Styles_Armenia.xlsx
+++ b/Informe_KPIs_CRM_ibis_Styles_Armenia.xlsx
@@ -5459,13 +5459,13 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>69623.5</v>
+        <v>69997.5</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>397.8</v>
+        <v>397.7</v>
       </c>
     </row>
     <row r="6">
@@ -5491,13 +5491,13 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>1148</v>
+        <v>774</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>382.7</v>
+        <v>387</v>
       </c>
     </row>
   </sheetData>

</xml_diff>